<commit_message>
Workflow and delivrable v5
</commit_message>
<xml_diff>
--- a/orthogonal_validation/DELIVERABLES/GSE130613_vs_Nanopore_v5_24:06/tables/step15_DE_overlap_Illumina_vs_Nanopore.xlsx
+++ b/orthogonal_validation/DELIVERABLES/GSE130613_vs_Nanopore_v5_24:06/tables/step15_DE_overlap_Illumina_vs_Nanopore.xlsx
@@ -441,16 +441,16 @@
   <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>